<commit_message>
Update September 14–20 substitutions and transfers
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="115">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -66,6 +66,303 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>14.09.2026, 5, 11:25-12:10, sala: 37</t>
+  </si>
+  <si>
+    <t>14.09.2026, 5, 11:25-12:10, sala: 41</t>
+  </si>
+  <si>
+    <t>Skarupa Agnieszka</t>
+  </si>
+  <si>
+    <t>5TH</t>
+  </si>
+  <si>
+    <t>Symulacyjna firma handlowa</t>
+  </si>
+  <si>
+    <t>14.09.2026, 6, 12:25-13:10, sala: 37</t>
+  </si>
+  <si>
+    <t>14.09.2026, 6, 12:25-13:10, sala: 41</t>
+  </si>
+  <si>
+    <t>14.09.2026, 7, 13:15-14:00, sala: 37</t>
+  </si>
+  <si>
+    <t>14.09.2026, 7, 13:15-14:00, sala: 41</t>
+  </si>
+  <si>
+    <t>14.09.2026, 8, 14:05-14:50, sala: 37</t>
+  </si>
+  <si>
+    <t>14.09.2026, 8, 14:05-14:50, sala: 41</t>
+  </si>
+  <si>
+    <t>15.09.2026, 2, 08:50-09:35, sala: 17</t>
+  </si>
+  <si>
+    <t>15.09.2026, 2, 08:50-09:35, sala: 22</t>
+  </si>
+  <si>
+    <t>Fiodorów Małgorzata</t>
+  </si>
+  <si>
+    <t>2WA|gr2</t>
+  </si>
+  <si>
+    <t>Język niemiecki</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona do sali 22</t>
+  </si>
+  <si>
+    <t>15.09.2026, 2, 08:50-09:35, sala: 26</t>
+  </si>
+  <si>
+    <t>15.09.2026, 2, 08:50-09:35, sala: 2</t>
+  </si>
+  <si>
+    <t>Hudziec Agnieszka</t>
+  </si>
+  <si>
+    <t>Chemia</t>
+  </si>
+  <si>
+    <t>przeniesienie lekcji do sali nr 2</t>
+  </si>
+  <si>
+    <t>Ulanowska Magdalena</t>
+  </si>
+  <si>
+    <t>1TFH</t>
+  </si>
+  <si>
+    <t>Język polski</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona do sali 17</t>
+  </si>
+  <si>
+    <t>15.09.2026, 2, 08:50-09:35, sala: 27</t>
+  </si>
+  <si>
+    <t>15.09.2026, 3, 09:40-10:25, sala: 27</t>
+  </si>
+  <si>
+    <t>Karczmarz Aleksandra</t>
+  </si>
+  <si>
+    <t>2TFA</t>
+  </si>
+  <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>15.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>15.09.2026, 7, 13:15-14:00, sala: 33</t>
+  </si>
+  <si>
+    <t>Galert Anna</t>
+  </si>
+  <si>
+    <t>1FB</t>
+  </si>
+  <si>
+    <t>15.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>15.09.2026, 8, 14:05-14:50, sala: 33</t>
+  </si>
+  <si>
+    <t>1CA|gr1</t>
+  </si>
+  <si>
+    <t>Język angielski</t>
+  </si>
+  <si>
+    <t>16.09.2026, 1, 08:00-08:45, sala: 32</t>
+  </si>
+  <si>
+    <t>16.09.2026, 1, 08:00-08:45, sala: 33</t>
+  </si>
+  <si>
+    <t>1TFH|gr1</t>
+  </si>
+  <si>
+    <t>przeniesienie do sali 33</t>
+  </si>
+  <si>
+    <t>16.09.2026, 1, 08:00-08:45, sala: sg6</t>
+  </si>
+  <si>
+    <t>16.09.2026, 1, 08:00-08:45, sala: 18</t>
+  </si>
+  <si>
+    <t>Pietrycha Małgorzata</t>
+  </si>
+  <si>
+    <t>1TH|DZ</t>
+  </si>
+  <si>
+    <t>Wychowanie fizyczne</t>
+  </si>
+  <si>
+    <t>przeniesienie do sali 18</t>
+  </si>
+  <si>
+    <t>16.09.2026, 2, 08:50-09:35, sala: 43</t>
+  </si>
+  <si>
+    <t>16.09.2026, 2, 08:50-09:35, sala: 33</t>
+  </si>
+  <si>
+    <t>Biezmienow Małgorzata</t>
+  </si>
+  <si>
+    <t>1TFH|gr2</t>
+  </si>
+  <si>
+    <t>16.09.2026, 2, 08:50-09:35, sala: sg6</t>
+  </si>
+  <si>
+    <t>16.09.2026, 2, 08:50-09:35, sala: 18</t>
+  </si>
+  <si>
+    <t>16.09.2026, 2, 08:50-09:35, sala: 23</t>
+  </si>
+  <si>
+    <t>2TFB</t>
+  </si>
+  <si>
+    <t>przeniesienie do sali 43</t>
+  </si>
+  <si>
+    <t>16.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>16.09.2026, 3, 09:40-10:25, sala: 3</t>
+  </si>
+  <si>
+    <t>Granatowska Mariola</t>
+  </si>
+  <si>
+    <t>2K|gr2</t>
+  </si>
+  <si>
+    <t>16.09.2026, 3, 09:40-10:25, sala: 19</t>
+  </si>
+  <si>
+    <t>Socha Dariusz</t>
+  </si>
+  <si>
+    <t>2S</t>
+  </si>
+  <si>
+    <t>Rozwój kompetencji zawodowych - kompetencje zawodowe</t>
+  </si>
+  <si>
+    <t>przeniesienie lekcji do sali 19</t>
+  </si>
+  <si>
+    <t>16.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>16.09.2026, 4, 10:35-11:20, sala: 2</t>
+  </si>
+  <si>
+    <t>4TH|gr2</t>
+  </si>
+  <si>
+    <t>16.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>16.09.2026, 5, 11:25-12:10, sala: bib</t>
+  </si>
+  <si>
+    <t>16.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>16.09.2026, 6, 12:25-13:10, sala: 2</t>
+  </si>
+  <si>
+    <t>3TFA</t>
+  </si>
+  <si>
+    <t>16.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>16.09.2026, 7, 13:15-14:00, sala: 2</t>
+  </si>
+  <si>
+    <t>2CB</t>
+  </si>
+  <si>
+    <t>17.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>17.09.2026, 3, 09:40-10:25, sala: 22</t>
+  </si>
+  <si>
+    <t>1FA|gr2</t>
+  </si>
+  <si>
+    <t>17.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>17.09.2026, 4, 10:35-11:20, sala: 22</t>
+  </si>
+  <si>
+    <t>1K|gr1</t>
+  </si>
+  <si>
+    <t>17.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>17.09.2026, 5, 11:25-12:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1FC|gr1</t>
+  </si>
+  <si>
+    <t>17.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>17.09.2026, 6, 12:25-13:10, sala: 3</t>
+  </si>
+  <si>
+    <t>1TFA|gr2</t>
+  </si>
+  <si>
+    <t>17.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>17.09.2026, 7, 13:15-14:00, sala: 33</t>
+  </si>
+  <si>
+    <t>1S|gr2</t>
+  </si>
+  <si>
+    <t>03.09.2026, 8, 14:05-14:50, sala: 3</t>
+  </si>
+  <si>
+    <t>18.09.2026, 4, 10:35-11:20, sala: 3</t>
+  </si>
+  <si>
+    <t>Jastrzębska-Majtyka Agnieszka</t>
+  </si>
+  <si>
+    <t>1FA</t>
+  </si>
+  <si>
+    <t>Techniki fryzjerskie</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona z 3 września 2026. Lekcja 4 sala 3</t>
   </si>
 </sst>
 </file>
@@ -515,7 +812,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{12e3485a-0ebb-4b5f-ab21-f76dd26e71c0}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{9ac8a8ec-ee10-4562-9495-7b065bd09d82}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -536,16 +833,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{fdeb3ec4-c6b1-48c0-ae06-77aed46fb4da}">
-  <dimension ref="A1:G2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f1ebbd62-7c32-4f8f-920f-b803558f5ad8}">
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="30.7142857142857" customWidth="1"/>
-    <col min="3" max="3" width="26.1428571428571" customWidth="1"/>
+    <col min="1" max="2" width="31.5714285714286" customWidth="1"/>
+    <col min="3" max="3" width="28.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="18.7142857142857" customWidth="1"/>
-    <col min="7" max="7" width="9.28571428571429" customWidth="1"/>
+    <col min="6" max="6" width="54.4285714285714" customWidth="1"/>
+    <col min="7" max="7" width="46.8571428571429" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="56.25" customHeight="1">
@@ -592,6 +889,627 @@
       </c>
       <c r="G2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15">
+      <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
+      <c r="A7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G8" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C15" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>68</v>
+      </c>
+      <c r="F15" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>62</v>
+      </c>
+      <c r="F16" t="s">
+        <v>63</v>
+      </c>
+      <c r="G16" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15">
+      <c r="A18" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F18" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" t="s">
+        <v>79</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" t="s">
+        <v>81</v>
+      </c>
+      <c r="G19" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15">
+      <c r="A20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" t="s">
+        <v>84</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>85</v>
+      </c>
+      <c r="F20" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15">
+      <c r="A21" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" t="s">
+        <v>87</v>
+      </c>
+      <c r="C21" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>85</v>
+      </c>
+      <c r="F21" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>90</v>
+      </c>
+      <c r="F22" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15">
+      <c r="A23" t="s">
+        <v>91</v>
+      </c>
+      <c r="B23" t="s">
+        <v>92</v>
+      </c>
+      <c r="C23" t="s">
+        <v>76</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>93</v>
+      </c>
+      <c r="F23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15">
+      <c r="A24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B24" t="s">
+        <v>95</v>
+      </c>
+      <c r="C24" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>96</v>
+      </c>
+      <c r="F24" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15">
+      <c r="A25" t="s">
+        <v>97</v>
+      </c>
+      <c r="B25" t="s">
+        <v>98</v>
+      </c>
+      <c r="C25" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>99</v>
+      </c>
+      <c r="F25" t="s">
+        <v>54</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15">
+      <c r="A26" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" t="s">
+        <v>49</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" t="s">
+        <v>54</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15">
+      <c r="A27" t="s">
+        <v>103</v>
+      </c>
+      <c r="B27" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" t="s">
+        <v>49</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>105</v>
+      </c>
+      <c r="F27" t="s">
+        <v>54</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15">
+      <c r="A28" t="s">
+        <v>106</v>
+      </c>
+      <c r="B28" t="s">
+        <v>107</v>
+      </c>
+      <c r="C28" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>108</v>
+      </c>
+      <c r="F28" t="s">
+        <v>54</v>
+      </c>
+      <c r="G28" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="15">
+      <c r="A29" t="s">
+        <v>109</v>
+      </c>
+      <c r="B29" t="s">
+        <v>110</v>
+      </c>
+      <c r="C29" t="s">
+        <v>111</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh September 14-20 substitutions and transfers
Import the updated exports for the same 14-20.09.2026 package: 109
substitutions, 38 transfers, 16 duty replacements and 4 other-activity
entries. Thursday gains four lesson changes and Friday is now filled in.

Diary names were removed with scripts/privacy_xlsx.py before the commit;
no other cell differs from the source export.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSteHAUcpUZjXBcPeyJY4A
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="143">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -245,15 +245,18 @@
     <t>16.09.2026, 3, 09:40-10:25, sala: 05</t>
   </si>
   <si>
+    <t>16.09.2026, 3, 09:40-10:25, sala: 23</t>
+  </si>
+  <si>
+    <t>Granatowska Mariola</t>
+  </si>
+  <si>
+    <t>2K|gr2</t>
+  </si>
+  <si>
     <t>16.09.2026, 3, 09:40-10:25, sala: 3</t>
   </si>
   <si>
-    <t>Granatowska Mariola</t>
-  </si>
-  <si>
-    <t>2K|gr2</t>
-  </si>
-  <si>
     <t>16.09.2026, 3, 09:40-10:25, sala: 19</t>
   </si>
   <si>
@@ -332,10 +335,25 @@
     <t>17.09.2026, 6, 12:25-13:10, sala: 05</t>
   </si>
   <si>
+    <t>17.09.2026, 6, 12:25-13:10, sala: 17</t>
+  </si>
+  <si>
+    <t>1TFA|gr2</t>
+  </si>
+  <si>
+    <t>17.09.2026, 10, 15:45-16:30, sala: 3</t>
+  </si>
+  <si>
     <t>17.09.2026, 6, 12:25-13:10, sala: 3</t>
   </si>
   <si>
-    <t>1TFA|gr2</t>
+    <t>Jastrzębska-Majtyka Agnieszka</t>
+  </si>
+  <si>
+    <t>4TFB</t>
+  </si>
+  <si>
+    <t>Projektowanie fryzur</t>
   </si>
   <si>
     <t>17.09.2026, 7, 13:15-14:00, sala: 05</t>
@@ -347,15 +365,33 @@
     <t>1S|gr2</t>
   </si>
   <si>
+    <t>18.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 2, 08:50-09:35, sala: 19</t>
+  </si>
+  <si>
+    <t>4TFA</t>
+  </si>
+  <si>
+    <t>18.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 3, 09:40-10:25, sala: 19</t>
+  </si>
+  <si>
+    <t>18.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 4, 10:35-11:20, sala: 19</t>
+  </si>
+  <si>
     <t>03.09.2026, 8, 14:05-14:50, sala: 3</t>
   </si>
   <si>
     <t>18.09.2026, 4, 10:35-11:20, sala: 3</t>
   </si>
   <si>
-    <t>Jastrzębska-Majtyka Agnieszka</t>
-  </si>
-  <si>
     <t>1FA</t>
   </si>
   <si>
@@ -363,6 +399,54 @@
   </si>
   <si>
     <t>lekcja przeniesiona z 3 września 2026. Lekcja 4 sala 3</t>
+  </si>
+  <si>
+    <t>18.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 5, 11:25-12:10, sala: 5</t>
+  </si>
+  <si>
+    <t>1TFB|gr1</t>
+  </si>
+  <si>
+    <t>18.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 6, 12:25-13:10, sala: 5</t>
+  </si>
+  <si>
+    <t>3TFB|gr1</t>
+  </si>
+  <si>
+    <t>18.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 7, 13:15-14:00, sala: 5</t>
+  </si>
+  <si>
+    <t>1CB|gr1</t>
+  </si>
+  <si>
+    <t>18.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 8, 14:05-14:50, sala: 5</t>
+  </si>
+  <si>
+    <t>18.09.2026, 9, 14:55-15:40, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 9, 14:55-15:40, sala: 18</t>
+  </si>
+  <si>
+    <t>18.09.2026, 10, 15:45-16:30, sala: 05</t>
+  </si>
+  <si>
+    <t>18.09.2026, 10, 15:45-16:30, sala: 2</t>
+  </si>
+  <si>
+    <t>1FB|gr1</t>
   </si>
 </sst>
 </file>
@@ -812,7 +896,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{9ac8a8ec-ee10-4562-9495-7b065bd09d82}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{20bdd12e-89f7-4a3b-91a8-f45b6eb69eb5}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -833,11 +917,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f1ebbd62-7c32-4f8f-920f-b803558f5ad8}">
-  <dimension ref="A1:G29"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f10504e1-0230-4624-ac2d-15b4fbaa712f}">
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="31.5714285714286" customWidth="1"/>
+    <col min="1" max="1" width="31.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="31.5714285714286" customWidth="1"/>
     <col min="3" max="3" width="28.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
@@ -1261,33 +1346,33 @@
     </row>
     <row r="19" spans="1:7" ht="15">
       <c r="A19" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="15">
       <c r="A20" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C20" t="s">
         <v>76</v>
@@ -1296,7 +1381,7 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F20" t="s">
         <v>54</v>
@@ -1307,10 +1392,10 @@
     </row>
     <row r="21" spans="1:7" ht="15">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C21" t="s">
         <v>76</v>
@@ -1319,7 +1404,7 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="F21" t="s">
         <v>54</v>
@@ -1330,10 +1415,10 @@
     </row>
     <row r="22" spans="1:7" ht="15">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C22" t="s">
         <v>76</v>
@@ -1342,7 +1427,7 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
         <v>54</v>
@@ -1353,10 +1438,10 @@
     </row>
     <row r="23" spans="1:7" ht="15">
       <c r="A23" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B23" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C23" t="s">
         <v>76</v>
@@ -1365,7 +1450,7 @@
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F23" t="s">
         <v>54</v>
@@ -1376,10 +1461,10 @@
     </row>
     <row r="24" spans="1:7" ht="15">
       <c r="A24" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B24" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C24" t="s">
         <v>49</v>
@@ -1388,7 +1473,7 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F24" t="s">
         <v>54</v>
@@ -1399,10 +1484,10 @@
     </row>
     <row r="25" spans="1:7" ht="15">
       <c r="A25" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C25" t="s">
         <v>49</v>
@@ -1411,7 +1496,7 @@
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F25" t="s">
         <v>54</v>
@@ -1422,10 +1507,10 @@
     </row>
     <row r="26" spans="1:7" ht="15">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" t="s">
         <v>49</v>
@@ -1434,7 +1519,7 @@
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F26" t="s">
         <v>54</v>
@@ -1445,10 +1530,10 @@
     </row>
     <row r="27" spans="1:7" ht="15">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B27" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C27" t="s">
         <v>49</v>
@@ -1457,7 +1542,7 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F27" t="s">
         <v>54</v>
@@ -1468,22 +1553,22 @@
     </row>
     <row r="28" spans="1:7" ht="15">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B28" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>109</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F28" t="s">
-        <v>54</v>
+        <v>111</v>
       </c>
       <c r="G28" t="s">
         <v>15</v>
@@ -1491,25 +1576,255 @@
     </row>
     <row r="29" spans="1:7" ht="15">
       <c r="A29" t="s">
+        <v>112</v>
+      </c>
+      <c r="B29" t="s">
+        <v>113</v>
+      </c>
+      <c r="C29" t="s">
+        <v>49</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>114</v>
+      </c>
+      <c r="F29" t="s">
+        <v>54</v>
+      </c>
+      <c r="G29" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="15">
+      <c r="A30" t="s">
+        <v>115</v>
+      </c>
+      <c r="B30" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" t="s">
+        <v>49</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>117</v>
+      </c>
+      <c r="F30" t="s">
+        <v>54</v>
+      </c>
+      <c r="G30" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="15">
+      <c r="A31" t="s">
+        <v>118</v>
+      </c>
+      <c r="B31" t="s">
+        <v>119</v>
+      </c>
+      <c r="C31" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>117</v>
+      </c>
+      <c r="F31" t="s">
+        <v>54</v>
+      </c>
+      <c r="G31" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="15">
+      <c r="A32" t="s">
+        <v>120</v>
+      </c>
+      <c r="B32" t="s">
+        <v>121</v>
+      </c>
+      <c r="C32" t="s">
+        <v>49</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>114</v>
+      </c>
+      <c r="F32" t="s">
+        <v>54</v>
+      </c>
+      <c r="G32" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="15">
+      <c r="A33" t="s">
+        <v>122</v>
+      </c>
+      <c r="B33" t="s">
+        <v>123</v>
+      </c>
+      <c r="C33" t="s">
         <v>109</v>
       </c>
-      <c r="B29" t="s">
-        <v>110</v>
-      </c>
-      <c r="C29" t="s">
-        <v>111</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>112</v>
-      </c>
-      <c r="F29" t="s">
-        <v>113</v>
-      </c>
-      <c r="G29" t="s">
-        <v>114</v>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F33" t="s">
+        <v>125</v>
+      </c>
+      <c r="G33" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="15">
+      <c r="A34" t="s">
+        <v>127</v>
+      </c>
+      <c r="B34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C34" t="s">
+        <v>49</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>129</v>
+      </c>
+      <c r="F34" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="15">
+      <c r="A35" t="s">
+        <v>130</v>
+      </c>
+      <c r="B35" t="s">
+        <v>131</v>
+      </c>
+      <c r="C35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>132</v>
+      </c>
+      <c r="F35" t="s">
+        <v>54</v>
+      </c>
+      <c r="G35" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="15">
+      <c r="A36" t="s">
+        <v>133</v>
+      </c>
+      <c r="B36" t="s">
+        <v>134</v>
+      </c>
+      <c r="C36" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>135</v>
+      </c>
+      <c r="F36" t="s">
+        <v>54</v>
+      </c>
+      <c r="G36" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="15">
+      <c r="A37" t="s">
+        <v>136</v>
+      </c>
+      <c r="B37" t="s">
+        <v>137</v>
+      </c>
+      <c r="C37" t="s">
+        <v>49</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>100</v>
+      </c>
+      <c r="F37" t="s">
+        <v>54</v>
+      </c>
+      <c r="G37" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="15">
+      <c r="A38" t="s">
+        <v>138</v>
+      </c>
+      <c r="B38" t="s">
+        <v>139</v>
+      </c>
+      <c r="C38" t="s">
+        <v>49</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>103</v>
+      </c>
+      <c r="F38" t="s">
+        <v>54</v>
+      </c>
+      <c r="G38" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="15">
+      <c r="A39" t="s">
+        <v>140</v>
+      </c>
+      <c r="B39" t="s">
+        <v>141</v>
+      </c>
+      <c r="C39" t="s">
+        <v>49</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>142</v>
+      </c>
+      <c r="F39" t="s">
+        <v>54</v>
+      </c>
+      <c r="G39" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Publish substitutions and transfers through 30 September
The new export widens the package from 14-20.09 to 14-30.09.2026: 179
substitutions, 42 transfers, 30 duty replacements and 7 other-activity
entries. Everything from the previous week is carried over unchanged; the
additions are 21-25.09 and 30.09, and one duty replacement on 17.09 is
gone from the source.

Seven diary names were removed with scripts/privacy_xlsx.py before the
commit; no other cell differs from the source export.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSteHAUcpUZjXBcPeyJY4A
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="154">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 14.09.2026 (pon.) - 20.09.2026 (niedz.)</t>
+    <t>Okres: 14.09.2026 (pon.) - 30.09.2026 (śr.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -365,6 +365,21 @@
     <t>1S|gr2</t>
   </si>
   <si>
+    <t>18.09.2026, 11, 16:35-17:20, sala: 44</t>
+  </si>
+  <si>
+    <t>17.09.2026, 11, 16:35-17:20, sala: 22</t>
+  </si>
+  <si>
+    <t>Staliś Donata</t>
+  </si>
+  <si>
+    <t>1B|gr2</t>
+  </si>
+  <si>
+    <t>p. Staliś, przeniesiony język angielski na czwartek 17.09.2026</t>
+  </si>
+  <si>
     <t>18.09.2026, 2, 08:50-09:35, sala: 05</t>
   </si>
   <si>
@@ -447,6 +462,24 @@
   </si>
   <si>
     <t>1FB|gr1</t>
+  </si>
+  <si>
+    <t>18.09.2026, 10, 15:45-16:30, sala: 44</t>
+  </si>
+  <si>
+    <t>22.09.2026, 9, 14:55-15:40, sala: 23</t>
+  </si>
+  <si>
+    <t>03.09.2026, 7, 13:15-14:00, sala: 3</t>
+  </si>
+  <si>
+    <t>25.09.2026, 4, 10:35-11:20, sala: 3</t>
+  </si>
+  <si>
+    <t>18.09.2026, 9, 14:55-15:40, sala: 44</t>
+  </si>
+  <si>
+    <t>29.09.2026, 9, 14:55-15:40, sala: 23</t>
   </si>
 </sst>
 </file>
@@ -896,7 +929,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{20bdd12e-89f7-4a3b-91a8-f45b6eb69eb5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{51ca9c1e-2b1d-44bc-8ac5-3d5dc8b208f6}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -917,17 +950,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f10504e1-0230-4624-ac2d-15b4fbaa712f}">
-  <dimension ref="A1:G39"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{388342d5-08c4-4acb-a066-3af7b3c98bba}">
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.7142857142857" customWidth="1"/>
-    <col min="2" max="2" width="31.5714285714286" customWidth="1"/>
+    <col min="1" max="2" width="31.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="28.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="54.4285714285714" customWidth="1"/>
-    <col min="7" max="7" width="46.8571428571429" customWidth="1"/>
+    <col min="7" max="7" width="54.1428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="56.25" customHeight="1">
@@ -1605,27 +1637,27 @@
         <v>116</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>117</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F30" t="s">
         <v>54</v>
       </c>
       <c r="G30" t="s">
-        <v>15</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="15">
       <c r="A31" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B31" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C31" t="s">
         <v>49</v>
@@ -1634,7 +1666,7 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="F31" t="s">
         <v>54</v>
@@ -1645,10 +1677,10 @@
     </row>
     <row r="32" spans="1:7" ht="15">
       <c r="A32" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B32" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C32" t="s">
         <v>49</v>
@@ -1657,7 +1689,7 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="F32" t="s">
         <v>54</v>
@@ -1668,25 +1700,25 @@
     </row>
     <row r="33" spans="1:7" ht="15">
       <c r="A33" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B33" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="C33" t="s">
-        <v>109</v>
+        <v>49</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="F33" t="s">
-        <v>125</v>
+        <v>54</v>
       </c>
       <c r="G33" t="s">
-        <v>126</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="15">
@@ -1697,7 +1729,7 @@
         <v>128</v>
       </c>
       <c r="C34" t="s">
-        <v>49</v>
+        <v>109</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
@@ -1706,18 +1738,18 @@
         <v>129</v>
       </c>
       <c r="F34" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="G34" t="s">
-        <v>15</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="15">
       <c r="A35" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B35" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C35" t="s">
         <v>49</v>
@@ -1726,7 +1758,7 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F35" t="s">
         <v>54</v>
@@ -1737,10 +1769,10 @@
     </row>
     <row r="36" spans="1:7" ht="15">
       <c r="A36" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B36" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C36" t="s">
         <v>49</v>
@@ -1749,7 +1781,7 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F36" t="s">
         <v>54</v>
@@ -1760,10 +1792,10 @@
     </row>
     <row r="37" spans="1:7" ht="15">
       <c r="A37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B37" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
@@ -1772,7 +1804,7 @@
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="F37" t="s">
         <v>54</v>
@@ -1783,10 +1815,10 @@
     </row>
     <row r="38" spans="1:7" ht="15">
       <c r="A38" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B38" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
@@ -1795,7 +1827,7 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F38" t="s">
         <v>54</v>
@@ -1806,10 +1838,10 @@
     </row>
     <row r="39" spans="1:7" ht="15">
       <c r="A39" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B39" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
@@ -1818,12 +1850,104 @@
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>142</v>
+        <v>103</v>
       </c>
       <c r="F39" t="s">
         <v>54</v>
       </c>
       <c r="G39" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="15">
+      <c r="A40" t="s">
+        <v>145</v>
+      </c>
+      <c r="B40" t="s">
+        <v>146</v>
+      </c>
+      <c r="C40" t="s">
+        <v>49</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>147</v>
+      </c>
+      <c r="F40" t="s">
+        <v>54</v>
+      </c>
+      <c r="G40" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="15">
+      <c r="A41" t="s">
+        <v>148</v>
+      </c>
+      <c r="B41" t="s">
+        <v>149</v>
+      </c>
+      <c r="C41" t="s">
+        <v>117</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>118</v>
+      </c>
+      <c r="F41" t="s">
+        <v>54</v>
+      </c>
+      <c r="G41" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="15">
+      <c r="A42" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" t="s">
+        <v>151</v>
+      </c>
+      <c r="C42" t="s">
+        <v>109</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>129</v>
+      </c>
+      <c r="F42" t="s">
+        <v>130</v>
+      </c>
+      <c r="G42" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="15">
+      <c r="A43" t="s">
+        <v>152</v>
+      </c>
+      <c r="B43" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" t="s">
+        <v>117</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>118</v>
+      </c>
+      <c r="F43" t="s">
+        <v>54</v>
+      </c>
+      <c r="G43" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Zaktualizuj zastępstwa i przeniesienia na okres 21-27.09.2026
Nowa paczka zawęża okres z 21.09-30.09 do 21.09-27.09.2026 i mocno
uzupełnia bieżący tydzień (22.09: 12->19, 23.09: 17->23, 24.09: 17->20,
25.09: 6->15 zastępstw).

- zastępstwa lekcyjne: 103
- przeniesienia: 13
- zastępstwa dyżurów: 22
- zajęcia inne: 0 (wszystkie 4 wpisy to nauczanie indywidualne)
- pominięte jako IND: 1 zastępstwo + 4 zajęcia inne

Dziennik zawiera już odwołanie lekcji Derezińskiej z 1B (21.09, lekcje
8-10), dodane wcześniej ręcznie — eksport przejmuje je bez zmian.

Wpisy na 28, 29 i 30.09 wypadają poza okres nowej paczki.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 21.09.2026 (pon.) - 30.09.2026 (śr.)</t>
+    <t>Okres: 21.09.2026 (pon.) - 27.09.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -113,6 +113,75 @@
     <t>Projektowanie fryzur</t>
   </si>
   <si>
+    <t>22.09.2026, 4, 10:35-11:20, sala: 09</t>
+  </si>
+  <si>
+    <t>22.09.2026, 4, 10:35-11:20, sala: 2</t>
+  </si>
+  <si>
+    <t>Leńczowska Iwona</t>
+  </si>
+  <si>
+    <t>3TFA</t>
+  </si>
+  <si>
+    <t>Rozwój kompetencji zawodowych - Fryzjerstwo naturalne</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona do sali 2</t>
+  </si>
+  <si>
+    <t>22.09.2026, 10, 15:45-16:30, sala: 30</t>
+  </si>
+  <si>
+    <t>22.09.2026, 5, 11:25-12:10, sala: 30</t>
+  </si>
+  <si>
+    <t>Filipek Anna</t>
+  </si>
+  <si>
+    <t>3CA</t>
+  </si>
+  <si>
+    <t>Język polski</t>
+  </si>
+  <si>
+    <t>22.09.2026, 7, 13:15-14:00, sala: 05</t>
+  </si>
+  <si>
+    <t>22.09.2026, 7, 13:15-14:00, sala: 27</t>
+  </si>
+  <si>
+    <t>1FB</t>
+  </si>
+  <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>22.09.2026, 6, 12:25-13:10, sala: 18</t>
+  </si>
+  <si>
+    <t>22.09.2026, 7, 13:15-14:00, sala: 18</t>
+  </si>
+  <si>
+    <t>Kaczorowski Waldemar</t>
+  </si>
+  <si>
+    <t>1CA</t>
+  </si>
+  <si>
+    <t>Historia</t>
+  </si>
+  <si>
+    <t>22.09.2026, 8, 14:05-14:50, sala: 05</t>
+  </si>
+  <si>
+    <t>22.09.2026, 8, 14:05-14:50, sala: 27</t>
+  </si>
+  <si>
+    <t>1CA|gr1</t>
+  </si>
+  <si>
     <t>18.09.2026, 10, 15:45-16:30, sala: 44</t>
   </si>
   <si>
@@ -165,18 +234,6 @@
   </si>
   <si>
     <t>lekcja przeniesiona z 3 września 2026. Lekcja 4 sala 3</t>
-  </si>
-  <si>
-    <t>21.09.2026, 8, 14:05-14:50, sala: 5</t>
-  </si>
-  <si>
-    <t>29.09.2026, 1, 08:00-08:45, sala: 3</t>
-  </si>
-  <si>
-    <t>18.09.2026, 9, 14:55-15:40, sala: 44</t>
-  </si>
-  <si>
-    <t>29.09.2026, 9, 14:55-15:40, sala: 23</t>
   </si>
 </sst>
 </file>
@@ -626,7 +683,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{13a8cd95-b1bd-4a81-8d9f-1abaa50bcdac}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e53389af-a0d1-4408-9f87-8b97dc84dc7e}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -647,8 +704,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{ec36a27a-87b5-4277-bb5a-ff264ec45518}">
-  <dimension ref="A1:G11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{457fcff3-d16b-4962-9674-b31f6bed98f1}">
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.7142857142857" customWidth="1"/>
@@ -792,99 +849,99 @@
         <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="15">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>39</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="15">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G9" t="s">
-        <v>48</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="15">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>53</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G10" t="s">
         <v>15</v>
@@ -892,25 +949,94 @@
     </row>
     <row r="11" spans="1:7" ht="15">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="F11" t="s">
         <v>20</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Dodaj przeniesienia na 29.09 (w tym Kopij, 3K)
Nowszy eksport przeniesień: 16 zamiast 13, nic nie ubyło. Dochodzą trzy
przeniesienia z celem 29.09:

- 3K, Edukacja obywatelska, Kopij Marcin: 22.09 lekcja 8 -> 29.09 lekcja 9
- 4TFA, Projektowanie fryzur, Krzemińska: 21.09 lekcja 8 -> 29.09 lekcja 1
- 1B|gr2, Język angielski, Staliś: 18.09 lekcja 9 -> 29.09 lekcja 9

Uwaga na rozjazd okresów: ten plik obejmuje 21.09-30.09, a opublikowany
plik zastępstw 21.09-27.09. Okno planu uczniowskiego liczy się z pliku
zastępstw, więc 29.09 pozostaje poza nim i cele tych trzech przeniesień
nie są tam klikalne. Lekcje źródłowe mają pełny opis z datą docelową.
Serwis nauczyciela pokazuje oba końce, bo jego okno to cały semestr.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="82">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 21.09.2026 (pon.) - 27.09.2026 (niedz.)</t>
+    <t>Okres: 21.09.2026 (pon.) - 30.09.2026 (śr.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -234,6 +234,36 @@
   </si>
   <si>
     <t>lekcja przeniesiona z 3 września 2026. Lekcja 4 sala 3</t>
+  </si>
+  <si>
+    <t>21.09.2026, 8, 14:05-14:50, sala: 5</t>
+  </si>
+  <si>
+    <t>29.09.2026, 1, 08:00-08:45, sala: 3</t>
+  </si>
+  <si>
+    <t>22.09.2026, 8, 14:05-14:50, sala: 19</t>
+  </si>
+  <si>
+    <t>29.09.2026, 9, 14:55-15:40, sala: 19</t>
+  </si>
+  <si>
+    <t>Kopij Marcin</t>
+  </si>
+  <si>
+    <t>3K</t>
+  </si>
+  <si>
+    <t>Edukacja obywatelska</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona na lekcję 9, wtorek 29.09.2026</t>
+  </si>
+  <si>
+    <t>18.09.2026, 9, 14:55-15:40, sala: 44</t>
+  </si>
+  <si>
+    <t>29.09.2026, 9, 14:55-15:40, sala: 23</t>
   </si>
 </sst>
 </file>
@@ -683,7 +713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e53389af-a0d1-4408-9f87-8b97dc84dc7e}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{99ed6e62-5f91-458d-8b33-4a1741ea94d9}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -704,8 +734,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{457fcff3-d16b-4962-9674-b31f6bed98f1}">
-  <dimension ref="A1:G14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e180d1af-f919-4420-a7e8-cd671590b933}">
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.7142857142857" customWidth="1"/>
@@ -1039,6 +1069,75 @@
         <v>71</v>
       </c>
     </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>30</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" t="s">
+        <v>74</v>
+      </c>
+      <c r="B16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>77</v>
+      </c>
+      <c r="F16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G16" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Zaktualizuj zastępstwa i przeniesienia na okres 21-30.09.2026
Eksport obejmuje wreszcie cały zakres obu plików (21.09-30.09), więc
domykają się dni 28-30.09, których poprzednia paczka nie miała.

- zastępstwa lekcyjne: 134
- przeniesienia: 16
- zastępstwa dyżurów: 28
- zajęcia inne: 0 (wszystkie 5 wpisów to nauczanie indywidualne)
- pominięte jako IND: 1 zastępstwo + 5 zajęć innych

Wobec opublikowanej paczki nic nie ubyło; doszło 31 zastępstw (głównie
28-30.09 i sześć na 22.09), 6 zmian dyżurów i 1 zajęcie inne.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -713,7 +713,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{99ed6e62-5f91-458d-8b33-4a1741ea94d9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{88291072-845a-4ed9-9663-c70a6aa97ea8}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -734,7 +734,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e180d1af-f919-4420-a7e8-cd671590b933}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e839826f-4b7e-4911-9a0e-397e51084c63}">
   <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Zaktualizuj zastępstwa i przeniesienia 21-30.09 (eksport 20/17)
Nic nie ubyło; 15 wpisów doprecyzowanych (sale, konkretni zastępcy
zamiast ogólnego "Zastępstwo"), doszło 42 zastępstw — głównie 28.09
(11 -> 31) i 30.09 (29 -> 49) — oraz 10 zmian dyżurów.

- zastępstwa lekcyjne: 356
- przeniesienia: 27
- zastępstwa dyżurów: 56
- zajęcia inne: 0
- pominięte jako IND: 1 zastępstwo + 5 zajęć innych

Plik przeniesień deklaruje okres do 01.10, ale żadne przeniesienie tam
nie celuje — lista jest identyczna jak w poprzedniej paczce.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -23,7 +23,7 @@
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 21.09.2026 (pon.) - 30.09.2026 (śr.)</t>
+    <t>Okres: 21.09.2026 (pon.) - 01.10.2026 (czw.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -806,7 +806,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{3e9fcfee-217f-49cb-8739-1fcc83fdc694}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d5093421-7288-47cb-b386-ebd5e3837843}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -827,7 +827,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d5eea1ed-6dcf-432c-9be5-5311c9298b34}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{10f8d696-d2dc-4a23-9df6-71e7f10ad98d}">
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Zaktualizuj eksport 21/18, zachowując korektę 3K kucharz 28.09
Nowy eksport różni się od opublikowanego jednym wierszem: dziennik zapisał
3K kucharz, 28.09, lekcja 2 jako zajęcia z wychowawcą u Agnieszki Skarupy
w sali 40. Decyzją użytkownika zostaje jego wersja: technologia
gastronomiczna, sala 41, "złączenie grup". Przejęta z dziennika jest tylko
forma płatności ("Bezpłatne" zamiast "-"), której korekta nie dotyczyła.

Nagłówek pliku przeniesień podaje teraz okres do 30.09 zamiast 01.10;
same przeniesienia bez zmian.

- zastępstwa lekcyjne: 356
- przeniesienia: 27
- zastępstwa dyżurów: 56
- zajęcia inne: 0
- pominięte jako IND: 1 zastępstwo + 5 zajęć innych

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PZStkgQc8MNG2spuAQPErL
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -23,7 +23,7 @@
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 21.09.2026 (pon.) - 01.10.2026 (czw.)</t>
+    <t>Okres: 21.09.2026 (pon.) - 30.09.2026 (śr.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -806,7 +806,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d5093421-7288-47cb-b386-ebd5e3837843}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{be605472-cd89-40dc-8757-cb2e73f9cea9}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -827,7 +827,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{10f8d696-d2dc-4a23-9df6-71e7f10ad98d}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{c148b9da-92f4-485d-8b58-b064abc5afde}">
   <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 28.09.2026–04.10.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="46">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -47,6 +47,72 @@
     <t>Uwagi</t>
   </si>
   <si>
+    <t>28.09.2026, 1, 08:00-08:45, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 1, 08:00-08:45, sala: 2</t>
+  </si>
+  <si>
+    <t>Karczmarz Aleksandra</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>2FC</t>
+  </si>
+  <si>
+    <t>Język angielski</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>28.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 2, 08:50-09:35, sala: 2</t>
+  </si>
+  <si>
+    <t>2K|gr1</t>
+  </si>
+  <si>
+    <t>28.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 3, 09:40-10:25, sala: 4</t>
+  </si>
+  <si>
+    <t>2FA</t>
+  </si>
+  <si>
+    <t>28.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 4, 10:35-11:20, sala: 4</t>
+  </si>
+  <si>
+    <t>2CA</t>
+  </si>
+  <si>
+    <t>28.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 5, 11:25-12:10, sala: 4</t>
+  </si>
+  <si>
+    <t>2S</t>
+  </si>
+  <si>
+    <t>28.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 6, 12:25-13:10, sala: 4</t>
+  </si>
+  <si>
+    <t>1TFH|gr1</t>
+  </si>
+  <si>
     <t>21.09.2026, 8, 14:05-14:50, sala: 5</t>
   </si>
   <si>
@@ -56,18 +122,12 @@
     <t>Krzemińska Beata</t>
   </si>
   <si>
-    <t>-</t>
-  </si>
-  <si>
     <t>4TFA</t>
   </si>
   <si>
     <t>Projektowanie fryzur</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>22.09.2026, 8, 14:05-14:50, sala: 19</t>
   </si>
   <si>
@@ -96,9 +156,6 @@
   </si>
   <si>
     <t>1B|gr2</t>
-  </si>
-  <si>
-    <t>Język angielski</t>
   </si>
 </sst>
 </file>
@@ -548,7 +605,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{29c1313f-3108-4ebb-956d-7674cb00d931}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{33f2d31d-3fb8-4bf8-acc5-66f774113371}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -569,12 +626,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{a9f28893-8915-4ee3-bf89-c5518e29ed6b}">
-  <dimension ref="A1:G4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{08261e5c-3230-461c-8f51-548c9bf8f4eb}">
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="30.7142857142857" customWidth="1"/>
-    <col min="3" max="3" width="19.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="20.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
     <col min="6" max="6" width="20.5714285714286" customWidth="1"/>
@@ -635,41 +692,179 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15">
+      <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="F4" t="s">
+      <c r="B6" t="s">
         <v>26</v>
       </c>
-      <c r="G4" t="s">
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15">
+      <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15">
+      <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>35</v>
+      </c>
+      <c r="G8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 05.10.2026–11.10.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -20,7 +20,7 @@
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 05.10.2026 (pon.) - 05.10.2026 (pon.)</t>
+    <t>Okres: 05.10.2026 (pon.) - 11.10.2026 (niedz.)</t>
   </si>
   <si>
     <t>Brak informacji o przeniesieniach</t>
@@ -464,7 +464,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{442cbf7f-1b47-40f4-8870-247c7124be7b}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{b2e56c85-98da-4065-a96d-87a99244f7fe}">
   <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 28.09.2026–11.10.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="108">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 05.10.2026 (pon.) - 11.10.2026 (niedz.)</t>
+    <t>Okres: 28.09.2026 (pon.) - 11.10.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -47,36 +47,231 @@
     <t>Uwagi</t>
   </si>
   <si>
+    <t>28.09.2026, 1, 08:00-08:45, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 1, 08:00-08:45, sala: 2</t>
+  </si>
+  <si>
+    <t>Karczmarz Aleksandra</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>2FC</t>
+  </si>
+  <si>
+    <t>Język angielski</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>28.09.2026, 2, 08:50-09:35, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 2, 08:50-09:35, sala: 2</t>
+  </si>
+  <si>
+    <t>2K|gr1</t>
+  </si>
+  <si>
+    <t>28.09.2026, 3, 09:40-10:25, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 3, 09:40-10:25, sala: 4</t>
+  </si>
+  <si>
+    <t>2FA</t>
+  </si>
+  <si>
+    <t>28.09.2026, 4, 10:35-11:20, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 4, 10:35-11:20, sala: 4</t>
+  </si>
+  <si>
+    <t>2CA</t>
+  </si>
+  <si>
+    <t>28.09.2026, 5, 11:25-12:10, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 5, 11:25-12:10, sala: 4</t>
+  </si>
+  <si>
+    <t>2S</t>
+  </si>
+  <si>
+    <t>28.09.2026, 6, 12:25-13:10, sala: 05</t>
+  </si>
+  <si>
+    <t>28.09.2026, 6, 12:25-13:10, sala: 4</t>
+  </si>
+  <si>
+    <t>1TFH|gr1</t>
+  </si>
+  <si>
+    <t>21.09.2026, 8, 14:05-14:50, sala: 5</t>
+  </si>
+  <si>
+    <t>29.09.2026, 1, 08:00-08:45, sala: 3</t>
+  </si>
+  <si>
+    <t>Krzemińska Beata</t>
+  </si>
+  <si>
+    <t>4TFA</t>
+  </si>
+  <si>
+    <t>Projektowanie fryzur</t>
+  </si>
+  <si>
+    <t>29.09.2026, 8, 14:05-14:50, sala: 34</t>
+  </si>
+  <si>
+    <t>29.09.2026, 7, 13:15-14:00, sala: 34</t>
+  </si>
+  <si>
+    <t>Kończyńska Małgorzata</t>
+  </si>
+  <si>
+    <t>3CB</t>
+  </si>
+  <si>
+    <t>Technika w produkcji cukierniczej</t>
+  </si>
+  <si>
+    <t>22.09.2026, 8, 14:05-14:50, sala: 19</t>
+  </si>
+  <si>
+    <t>29.09.2026, 9, 14:55-15:40, sala: 19</t>
+  </si>
+  <si>
+    <t>Kopij Marcin</t>
+  </si>
+  <si>
+    <t>3K</t>
+  </si>
+  <si>
+    <t>Edukacja obywatelska</t>
+  </si>
+  <si>
+    <t>lekcja przeniesiona na lekcję 9, wtorek 29.09.2026</t>
+  </si>
+  <si>
+    <t>18.09.2026, 9, 14:55-15:40, sala: 44</t>
+  </si>
+  <si>
+    <t>29.09.2026, 9, 14:55-15:40, sala: 23</t>
+  </si>
+  <si>
+    <t>Staliś Donata</t>
+  </si>
+  <si>
+    <t>1B|gr2</t>
+  </si>
+  <si>
+    <t>30.09.2026, 8, 14:05-14:50, sala: sg5</t>
+  </si>
+  <si>
+    <t>30.09.2026, 5, 11:25-12:10, sala: sg5</t>
+  </si>
+  <si>
+    <t>Dalach Krystyna</t>
+  </si>
+  <si>
+    <t>Wychowanie fizyczne</t>
+  </si>
+  <si>
+    <t>30.09.2026, 8, 14:05-14:50, sala: 22</t>
+  </si>
+  <si>
+    <t>30.09.2026, 5, 11:25-12:10, sala: 22</t>
+  </si>
+  <si>
+    <t>Ulanowska Magdalena</t>
+  </si>
+  <si>
+    <t>1FC</t>
+  </si>
+  <si>
+    <t>Język polski</t>
+  </si>
+  <si>
+    <t>30.09.2026, 1, 08:00-08:45, sala: 4</t>
+  </si>
+  <si>
+    <t>30.09.2026, 6, 12:25-13:10, sala: 4</t>
+  </si>
+  <si>
+    <t>Kruk Marcin</t>
+  </si>
+  <si>
+    <t>Techniki fryzjerskie</t>
+  </si>
+  <si>
+    <t>30.09.2026, 1, 08:00-08:45, sala: 2</t>
+  </si>
+  <si>
+    <t>30.09.2026, 6, 12:25-13:10, sala: 2</t>
+  </si>
+  <si>
+    <t>Leńczowska Iwona</t>
+  </si>
+  <si>
+    <t>01.10.2026, 10, 15:45-16:30, sala: 41</t>
+  </si>
+  <si>
+    <t>01.10.2026, 6, 12:25-13:10, sala: 41</t>
+  </si>
+  <si>
+    <t>Czukiewska Bożena</t>
+  </si>
+  <si>
+    <t>2TH</t>
+  </si>
+  <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>02.10.2026, 2, 08:50-09:35, sala: 17</t>
+  </si>
+  <si>
+    <t>02.10.2026, 3, 09:40-10:25, sala: 17</t>
+  </si>
+  <si>
+    <t>Nestoruk Lidia</t>
+  </si>
+  <si>
+    <t>02.10.2026, 10, 15:45-16:30, sala: 23</t>
+  </si>
+  <si>
+    <t>02.10.2026, 10, 15:45-16:30, sala: 22</t>
+  </si>
+  <si>
+    <t>Biczysko Wojciech</t>
+  </si>
+  <si>
+    <t>1TFH</t>
+  </si>
+  <si>
+    <t>Fizyka</t>
+  </si>
+  <si>
     <t>05.10.2026, 1, 08:00-08:45, sala: 05</t>
   </si>
   <si>
     <t>05.10.2026, 1, 08:00-08:45, sala: 2</t>
   </si>
   <si>
-    <t>Karczmarz Aleksandra</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>2FC</t>
-  </si>
-  <si>
-    <t>Język angielski</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>05.10.2026, 2, 08:50-09:35, sala: 05</t>
   </si>
   <si>
     <t>05.10.2026, 2, 08:50-09:35, sala: 2</t>
   </si>
   <si>
-    <t>2K|gr1</t>
-  </si>
-  <si>
     <t>05.10.2026, 3, 09:40-10:25, sala: 32</t>
   </si>
   <si>
@@ -95,36 +290,24 @@
     <t>05.10.2026, 3, 09:40-10:25, sala: 4</t>
   </si>
   <si>
-    <t>2FA</t>
-  </si>
-  <si>
     <t>05.10.2026, 4, 10:35-11:20, sala: 05</t>
   </si>
   <si>
     <t>05.10.2026, 4, 10:35-11:20, sala: 4</t>
   </si>
   <si>
-    <t>2CA</t>
-  </si>
-  <si>
     <t>05.10.2026, 5, 11:25-12:10, sala: 05</t>
   </si>
   <si>
     <t>05.10.2026, 5, 11:25-12:10, sala: 4</t>
   </si>
   <si>
-    <t>2S</t>
-  </si>
-  <si>
     <t>05.10.2026, 6, 12:25-13:10, sala: 05</t>
   </si>
   <si>
     <t>05.10.2026, 6, 12:25-13:10, sala: 4</t>
   </si>
   <si>
-    <t>1TFH|gr1</t>
-  </si>
-  <si>
     <t>05.10.2026, 8, 14:05-14:50, sala: 43</t>
   </si>
   <si>
@@ -135,6 +318,30 @@
   </si>
   <si>
     <t>1CA|gr2</t>
+  </si>
+  <si>
+    <t>06.10.2026, 8, 14:05-14:50, sala: 5</t>
+  </si>
+  <si>
+    <t>06.10.2026, 1, 08:00-08:45, sala: 3</t>
+  </si>
+  <si>
+    <t>Zajęcia praktyczne - projektowanie i wykonywanie fryzur</t>
+  </si>
+  <si>
+    <t>09.10.2026, 12, 17:25-18:10, sala: 37</t>
+  </si>
+  <si>
+    <t>06.10.2026, 9, 14:55-15:40, sala: 37</t>
+  </si>
+  <si>
+    <t>Młynarczyk Paweł</t>
+  </si>
+  <si>
+    <t>3B</t>
+  </si>
+  <si>
+    <t>Informatyka</t>
   </si>
 </sst>
 </file>
@@ -584,7 +791,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{76d477c4-6d8a-40db-a17d-e33b1fb429d5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{c3db1c9b-3531-4658-9988-3412d045ddd7}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -605,16 +812,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{2d2f9bd4-300a-4e8b-b7b6-183d6cadc510}">
-  <dimension ref="A1:G9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{4530ac15-6637-4148-a817-f402b9544e78}">
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="30.7142857142857" customWidth="1"/>
+    <col min="1" max="2" width="31.7142857142857" customWidth="1"/>
     <col min="3" max="3" width="22.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="14.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="9.28571428571429" customWidth="1"/>
+    <col min="6" max="6" width="51.1428571428571" customWidth="1"/>
+    <col min="7" max="7" width="44.7142857142857" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="56.25" customHeight="1">
@@ -694,13 +901,13 @@
         <v>20</v>
       </c>
       <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
       </c>
       <c r="F4" t="s">
         <v>14</v>
@@ -711,10 +918,10 @@
     </row>
     <row r="5" spans="1:7" ht="15">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -723,7 +930,7 @@
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
         <v>14</v>
@@ -734,10 +941,10 @@
     </row>
     <row r="6" spans="1:7" ht="15">
       <c r="A6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>27</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -746,7 +953,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
@@ -757,10 +964,10 @@
     </row>
     <row r="7" spans="1:7" ht="15">
       <c r="A7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" t="s">
         <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -769,7 +976,7 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
         <v>14</v>
@@ -780,13 +987,13 @@
     </row>
     <row r="8" spans="1:7" ht="15">
       <c r="A8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
@@ -795,7 +1002,7 @@
         <v>34</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="G8" t="s">
         <v>15</v>
@@ -803,24 +1010,461 @@
     </row>
     <row r="9" spans="1:7" ht="15">
       <c r="A9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15">
+      <c r="A10" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>44</v>
+      </c>
+      <c r="F10" t="s">
+        <v>45</v>
+      </c>
+      <c r="G10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
         <v>14</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15">
+      <c r="A12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>60</v>
+      </c>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" t="s">
+        <v>62</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>58</v>
+      </c>
+      <c r="F14" t="s">
+        <v>63</v>
+      </c>
+      <c r="G14" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15">
+      <c r="A15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s">
+        <v>63</v>
+      </c>
+      <c r="G15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15">
+      <c r="A16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
+        <v>69</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B17" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" t="s">
+        <v>71</v>
+      </c>
+      <c r="G17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15">
+      <c r="A18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" t="s">
+        <v>76</v>
+      </c>
+      <c r="C18" t="s">
+        <v>77</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" t="s">
+        <v>79</v>
+      </c>
+      <c r="G18" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15">
+      <c r="A19" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15">
+      <c r="A20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15">
+      <c r="A21" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15">
+      <c r="A22" t="s">
+        <v>88</v>
+      </c>
+      <c r="B22" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15">
+      <c r="A23" t="s">
+        <v>90</v>
+      </c>
+      <c r="B23" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="15">
+      <c r="A24" t="s">
+        <v>92</v>
+      </c>
+      <c r="B24" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>27</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="15">
+      <c r="A25" t="s">
+        <v>94</v>
+      </c>
+      <c r="B25" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>30</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="15">
+      <c r="A26" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" t="s">
+        <v>97</v>
+      </c>
+      <c r="C26" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="15">
+      <c r="A27" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" t="s">
+        <v>101</v>
+      </c>
+      <c r="C27" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>34</v>
+      </c>
+      <c r="F27" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="15">
+      <c r="A28" t="s">
+        <v>103</v>
+      </c>
+      <c r="B28" t="s">
+        <v>104</v>
+      </c>
+      <c r="C28" t="s">
+        <v>105</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" t="s">
+        <v>107</v>
+      </c>
+      <c r="G28" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 12.10.2026–18.10.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -575,7 +575,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{8501e6e8-b671-4e51-923c-fcb2ce468205}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{135b3677-0e40-4294-989a-eecd201cfa42}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -596,7 +596,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{71d32433-5468-46d4-9263-c813cb2ea8a2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{d445d90c-5536-4f67-8eda-7b8c649d0418}">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 19.10.2026–25.10.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="42">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 12.10.2026 (pon.) - 18.10.2026 (niedz.)</t>
+    <t>Okres: 19.10.2026 (pon.) - 25.10.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -47,139 +47,103 @@
     <t>Uwagi</t>
   </si>
   <si>
-    <t>12.10.2026, 1, 08:00-08:45, sala: 05</t>
-  </si>
-  <si>
-    <t>12.10.2026, 1, 08:00-08:45, sala: 4</t>
-  </si>
-  <si>
-    <t>Karczmarz Aleksandra</t>
+    <t>19.10.2026, 4, 10:35-11:20, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 1, 08:00-08:45, sala: prf2</t>
+  </si>
+  <si>
+    <t>Jaworska Edyta</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t>2FC</t>
-  </si>
-  <si>
-    <t>Język angielski</t>
+    <t>2TFA|gr2</t>
+  </si>
+  <si>
+    <t>Zajęcia praktyczne - wykonywanie usług fryzjerskich</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>12.10.2026, 2, 08:50-09:35, sala: 05</t>
-  </si>
-  <si>
-    <t>12.10.2026, 2, 08:50-09:35, sala: 2</t>
-  </si>
-  <si>
-    <t>2K|gr1</t>
-  </si>
-  <si>
-    <t>12.10.2026, 9, 14:55-15:40, sala: 31</t>
-  </si>
-  <si>
-    <t>12.10.2026, 2, 08:50-09:35, sala: 31</t>
-  </si>
-  <si>
-    <t>Sałdyka-Rusek Karolina</t>
-  </si>
-  <si>
-    <t>2S</t>
-  </si>
-  <si>
-    <t>Edukacja zdrowotna</t>
-  </si>
-  <si>
-    <t>12.10.2026, 3, 09:40-10:25, sala: 32</t>
-  </si>
-  <si>
-    <t>12.10.2026, 3, 09:40-10:25, sala: 17</t>
-  </si>
-  <si>
-    <t>Biezmienow Małgorzata</t>
-  </si>
-  <si>
-    <t>1FB|gr2</t>
-  </si>
-  <si>
-    <t>12.10.2026, 3, 09:40-10:25, sala: 05</t>
-  </si>
-  <si>
-    <t>12.10.2026, 3, 09:40-10:25, sala: 4</t>
-  </si>
-  <si>
-    <t>2FA</t>
-  </si>
-  <si>
-    <t>12.10.2026, 4, 10:35-11:20, sala: 40</t>
-  </si>
-  <si>
-    <t>12.10.2026, 4, 10:35-11:20, sala: 26</t>
-  </si>
-  <si>
-    <t>Mocarski Arkadiusz</t>
-  </si>
-  <si>
-    <t>2K</t>
-  </si>
-  <si>
-    <t>Rozwój kompetencji zawodowych - Zasady zdrowego żywienia</t>
-  </si>
-  <si>
-    <t>12.10.2026, 5, 11:25-12:10, sala: 05</t>
-  </si>
-  <si>
-    <t>12.10.2026, 5, 11:25-12:10, sala: 4</t>
-  </si>
-  <si>
-    <t>12.10.2026, 5, 11:25-12:10, sala: 40</t>
-  </si>
-  <si>
-    <t>12.10.2026, 5, 11:25-12:10, sala: 26</t>
-  </si>
-  <si>
-    <t>12.10.2026, 6, 12:25-13:10, sala: 05</t>
-  </si>
-  <si>
-    <t>12.10.2026, 6, 12:25-13:10, sala: 4</t>
-  </si>
-  <si>
-    <t>1TFH|gr1</t>
-  </si>
-  <si>
-    <t>15.10.2026, 1, 08:00-08:45, sala: sg1</t>
-  </si>
-  <si>
-    <t>15.10.2026, 4, 10:35-11:20, sala: sg1</t>
-  </si>
-  <si>
-    <t>Rejno Julita</t>
-  </si>
-  <si>
-    <t>3CB</t>
-  </si>
-  <si>
-    <t>Wychowanie fizyczne</t>
+    <t>19.10.2026, 10, 15:45-16:30, sala: 6</t>
+  </si>
+  <si>
+    <t>19.10.2026, 1, 08:00-08:45, sala: 6</t>
+  </si>
+  <si>
+    <t>Sobczak Anna</t>
+  </si>
+  <si>
+    <t>2TFA|gr1</t>
+  </si>
+  <si>
+    <t>19.10.2026, 5, 11:25-12:10, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 2, 08:50-09:35, sala: prf2</t>
+  </si>
+  <si>
+    <t>16.10.2026, 5, 11:25-12:10, sala: 33</t>
   </si>
   <si>
     <t>19.10.2026, 2, 08:50-09:35, sala: 33</t>
   </si>
   <si>
-    <t>16.10.2026, 5, 11:25-12:10, sala: 33</t>
-  </si>
-  <si>
     <t>Krycia Ewelina</t>
   </si>
   <si>
     <t>1TFA</t>
   </si>
   <si>
+    <t>Zajęcia z wychowawcą</t>
+  </si>
+  <si>
+    <t>przeniesienie lekcji na poniedziałek 19.10.2026</t>
+  </si>
+  <si>
+    <t>19.10.2026, 9, 14:55-15:40, sala: 6</t>
+  </si>
+  <si>
+    <t>19.10.2026, 2, 08:50-09:35, sala: 6</t>
+  </si>
+  <si>
+    <t>19.10.2026, 6, 12:25-13:10, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 3, 09:40-10:25, sala: prf2</t>
+  </si>
+  <si>
+    <t>23.10.2026, 5, 11:25-12:10, sala: 33</t>
+  </si>
+  <si>
+    <t>19.10.2026, 3, 09:40-10:25, sala: 33</t>
+  </si>
+  <si>
+    <t>19.10.2026, 8, 14:05-14:50, sala: 6</t>
+  </si>
+  <si>
+    <t>19.10.2026, 3, 09:40-10:25, sala: 6</t>
+  </si>
+  <si>
+    <t>19.10.2026, 7, 13:15-14:00, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 8, 14:05-14:50, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 9, 14:55-15:40, sala: prf2</t>
+  </si>
+  <si>
+    <t>19.10.2026, 10, 15:45-16:30, sala: prf2</t>
+  </si>
+  <si>
     <t>Język polski</t>
   </si>
   <si>
-    <t>przeniesienie lekcji na piątek 16.10.2026</t>
+    <t>przeniesienie lekcji na piątek 23.10.2026</t>
   </si>
 </sst>
 </file>
@@ -629,7 +593,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{09f4da6c-49c5-474c-ae63-5bbe07619aa1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{935dc65c-a2f3-4356-a9d4-b485bfb6789f}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -650,16 +614,17 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{e3fd7afd-c90f-44f0-98fd-37aa07e4d1a6}">
-  <dimension ref="A1:G12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{fd80e5de-4ebe-48f2-9583-00b9be78f857}">
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="31.5714285714286" customWidth="1"/>
-    <col min="3" max="3" width="22.4285714285714" customWidth="1"/>
+    <col min="1" max="1" width="33.2857142857143" customWidth="1"/>
+    <col min="2" max="2" width="32.2857142857143" customWidth="1"/>
+    <col min="3" max="3" width="19.4285714285714" customWidth="1"/>
     <col min="4" max="4" width="32.7142857142857" customWidth="1"/>
     <col min="5" max="5" width="10.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="56.1428571428571" customWidth="1"/>
-    <col min="7" max="7" width="36.7142857142857" customWidth="1"/>
+    <col min="6" max="6" width="46.8571428571429" customWidth="1"/>
+    <col min="7" max="7" width="42.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="56.25" customHeight="1">
@@ -716,13 +681,13 @@
         <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
         <v>14</v>
@@ -733,22 +698,22 @@
     </row>
     <row r="4" spans="1:7" ht="15">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="F4" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
@@ -756,25 +721,25 @@
     </row>
     <row r="5" spans="1:7" ht="15">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" t="s">
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
         <v>25</v>
       </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>26</v>
       </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>27</v>
-      </c>
-      <c r="F5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="15">
@@ -785,13 +750,13 @@
         <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
         <v>14</v>
@@ -802,22 +767,22 @@
     </row>
     <row r="7" spans="1:7" ht="15">
       <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" t="s">
         <v>31</v>
       </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="F7" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="G7" t="s">
         <v>15</v>
@@ -825,45 +790,45 @@
     </row>
     <row r="8" spans="1:7" ht="15">
       <c r="A8" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="15">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="C9" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="G9" t="s">
         <v>15</v>
@@ -871,10 +836,10 @@
     </row>
     <row r="10" spans="1:7" ht="15">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>9</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -883,7 +848,7 @@
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="F10" t="s">
         <v>14</v>
@@ -894,22 +859,22 @@
     </row>
     <row r="11" spans="1:7" ht="15">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
+        <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="F11" t="s">
-        <v>47</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
         <v>15</v>
@@ -917,25 +882,71 @@
     </row>
     <row r="12" spans="1:7" ht="15">
       <c r="A12" t="s">
-        <v>48</v>
+        <v>38</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="F12" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>53</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15">
+      <c r="A14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
+      <c r="C14" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Aktualizacja zastępstw i przeniesień 26.10.2026–01.11.2026
Oczyszczone eksporty z dziennika wgrane przez stronę aktualizacji (adeodatus11).
</commit_message>
<xml_diff>
--- a/InformacjeOPrzeniesieniach.xlsx
+++ b/InformacjeOPrzeniesieniach.xlsx
@@ -18,12 +18,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="44">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
   <si>
-    <t>Okres: 26.10.2026 (pon.) - 31.10.2026 (sob.)</t>
+    <t>Okres: 26.10.2026 (pon.) - 01.11.2026 (niedz.)</t>
   </si>
   <si>
     <t>Przeniesiono z</t>
@@ -117,6 +117,24 @@
   </si>
   <si>
     <t>p. Socha, przeniesienie lekcji z 8 godziny</t>
+  </si>
+  <si>
+    <t>27.10.2026, 8, 14:05-14:50, sala: 34</t>
+  </si>
+  <si>
+    <t>29.10.2026, 9, 14:55-15:40, sala: 34</t>
+  </si>
+  <si>
+    <t>Kończyńska Małgorzata</t>
+  </si>
+  <si>
+    <t>3CB</t>
+  </si>
+  <si>
+    <t>Technika w produkcji cukierniczej</t>
+  </si>
+  <si>
+    <t>przeniesiona na 29.10.2026 lekcja 9</t>
   </si>
   <si>
     <t>30.10.2026, 3, 09:40-10:25, sala: 31</t>
@@ -581,7 +599,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{91b82e9e-64e1-4bf3-900e-6fdfd9c6852d}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f2761a2e-9f70-4688-8f75-81e632dff730}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -602,8 +620,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{ba5d60c2-d81e-431d-a0a2-d4ab28cea166}">
-  <dimension ref="A1:G8"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{2dda2867-5fe5-4ed6-97f7-2d64e434d920}">
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="33.2857142857143" customWidth="1"/>
@@ -796,6 +814,29 @@
         <v>37</v>
       </c>
       <c r="G8" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15">
+      <c r="A9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" t="s">
         <v>15</v>
       </c>
     </row>

</xml_diff>